<commit_message>
data: unify survey and expert item ids on canonical code keys
</commit_message>
<xml_diff>
--- a/validation/expert-study/expert_rating_form_R3.xlsx
+++ b/validation/expert-study/expert_rating_form_R3.xlsx
@@ -783,7 +783,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>app_domain_boundary</t>
+          <t>A5</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -807,7 +807,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>app_resilience_pattern</t>
+          <t>A6</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -1647,7 +1647,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>governance_control_matrix</t>
+          <t>AGD6</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -1671,7 +1671,7 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>governance_decision_log</t>
+          <t>AGD7</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -1695,7 +1695,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>infra_recovery</t>
+          <t>DIN5</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -1719,7 +1719,7 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>infra_scalability</t>
+          <t>DIN6</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -1743,7 +1743,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>integration_contract</t>
+          <t>IP7</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -1767,7 +1767,7 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>integration_dependency_map</t>
+          <t>IP8</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -2055,7 +2055,7 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>security_identity_access</t>
+          <t>SCR11</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">

</xml_diff>

<commit_message>
data: align fixture and survey labels to canonical catalog names
</commit_message>
<xml_diff>
--- a/validation/expert-study/expert_rating_form_R3.xlsx
+++ b/validation/expert-study/expert_rating_form_R3.xlsx
@@ -793,7 +793,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Application</t>
+          <t>Context &amp; Application</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -812,12 +812,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Application Resilience Pattern</t>
+          <t>Application Resilience</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Application</t>
+          <t>Context &amp; Application</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -1657,7 +1657,7 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Governance</t>
+          <t>Architecture Governance &amp; Decision</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -1681,7 +1681,7 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Governance</t>
+          <t>Architecture Governance &amp; Decision</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -1705,7 +1705,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
+          <t>Deployment / Infrastructure / Networking</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -1729,7 +1729,7 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
+          <t>Deployment / Infrastructure / Networking</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -1753,7 +1753,7 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Integration</t>
+          <t>Integration &amp; Processing</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -1777,7 +1777,7 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Integration</t>
+          <t>Integration &amp; Processing</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -2065,7 +2065,7 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Security, Compliance &amp; Risk</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">

</xml_diff>